<commit_message>
D2b: DeepSeek-drafted candidate responses, screened and annotated by the researcher
- d2b_generate.py: DeepSeek plays a learner; sees only the problem text and a plain description
  of the response wanted (never rules, codes or the reference solution); fills response columns
  only, rows shuffled; drafting intention kept in eval/d2b_generation_log.json, not the workbook
- d2b_import.py records response_origin (llm_generated / llm_edited / researcher_written);
  eval_diagnosis_d2b.py reports results by origin
- evaluation_plan V1.2: §4.2 amendment, §9 threat, change log
</commit_message>
<xml_diff>
--- a/eval/d2b_cases.xlsx
+++ b/eval/d2b_cases.xlsx
@@ -2307,7 +2307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:B57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2419,504 +2419,516 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr"/>
-      <c r="B11" s="3" t="inlineStr"/>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>用 DeepSeek 生成候选作答时（python scripts/d2b_generate.py）：逐条看，不像真实学生的删掉或改写，然后像自己写的一样独立标注。生成意图存在 eval/d2b_generation_log.json，标注完成并冻结之前不要打开它。</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>数据集必须包含（评估计划 §4.2，导入时会自动检查）</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>总数</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>40–60 条</t>
-        </is>
-      </c>
+      <c r="B13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>E1–E7</t>
+          <t>总数</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>每个类别至少 5 条（按 primary_error 计）</t>
+          <t>40–60 条</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>正确作答</t>
+          <t>E1–E7</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>占 20–30%：包括等价方程、另一种设法、另一种解法、只写对最终答案 — 用 tags 标 equivalent_equation / alt_definition / alt_working</t>
+          <t>每个类别至少 5 条（按 primary_error 计）</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>正确作答</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>至少 5 条（reference_status = uncertain）</t>
+          <t>占 20–30%：包括等价方程、另一种设法、另一种解法、只写对最终答案 — 用 tags 标 equivalent_equation / alt_definition / alt_working</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>记号有歧义</t>
+          <t>uncertain</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>至少 3 条，例如 1/3x — tags 标 ambiguous_notation</t>
+          <t>至少 5 条（reference_status = uncertain）</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>只有最终答案且不对</t>
+          <t>记号有歧义</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>至少 5 条（layer = answer，reference_status 不是 correct）</t>
+          <t>至少 3 条，例如 1/3x — tags 标 ambiguous_notation</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>多个错误</t>
+          <t>只有最终答案且不对</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>至少 5 条（secondary_errors 不为空）</t>
+          <t>至少 5 条（layer = answer，reference_status 不是 correct）</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>逐行解方程</t>
+          <t>多个错误</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>至少 10 条（layer = execution，且填了 first_invalid_step）</t>
+          <t>至少 5 条（secondary_errors 不为空）</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
+          <t>逐行解方程</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>至少 10 条（layer = execution，且填了 first_invalid_step）</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
           <t>第二标注人</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>至少 20% 由另一个人盲标（python scripts/d2b_second.py export）</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr"/>
-      <c r="B22" s="3" t="inlineStr"/>
-    </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>错误类别（详见 docs/error_taxonomy.md）</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>E1</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>没读懂题目要求什么（求错了量）</t>
-        </is>
-      </c>
+      <c r="B24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>未知数定义不清或前后不一致</t>
+          <t>没读懂题目要求什么（求错了量）</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>数量关系错误</t>
+          <t>未知数定义不清或前后不一致</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>中文表述翻译成数学时的固定错误（E4-01 比…多 方向反 … E4-08 少了三分之一）</t>
+          <t>数量关系错误</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>E5</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>单位或数量级错误</t>
+          <t>中文表述翻译成数学时的固定错误（E4-01 比…多 方向反 … E4-08 少了三分之一）</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>E5</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>算术计算错误</t>
+          <t>单位或数量级错误</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
+          <t>E6</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>算术计算错误</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
           <t>E7</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>代数变形或符号错误（移项不变号、去括号等）</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr"/>
-      <c r="B31" s="3" t="inlineStr"/>
-    </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr"/>
+      <c r="B32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>填完之后</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>检查</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>python scripts/d2b_import.py --check</t>
-        </is>
-      </c>
+      <c r="B33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>导入</t>
+          <t>检查</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>python scripts/d2b_import.py</t>
+          <t>python scripts/d2b_import.py --check</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>第二标注人</t>
+          <t>导入</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>python scripts/d2b_second.py export   然后   python scripts/d2b_second.py compare</t>
+          <t>python scripts/d2b_import.py</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>冻结</t>
+          <t>第二标注人</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>所有 review_status = reviewed 后提交：git add eval  → git commit → git push</t>
+          <t>python scripts/d2b_second.py export   然后   python scripts/d2b_second.py compare</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
+          <t>冻结</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>所有 review_status = reviewed 后提交：git add eval  → git commit → git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
           <t>运行</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>python scripts/eval_diagnosis_d2b.py            （默认只跑 test，70%）</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr"/>
-      <c r="B38" s="3" t="inlineStr"/>
-    </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr"/>
+      <c r="B39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>列说明</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>case_id</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>编号，已预填 D2b-001…；不用的行留着即可（没有 question_id 的行会被跳过）</t>
-        </is>
-      </c>
+      <c r="B40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>question_id</t>
+          <t>case_id</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>对应题库哪一题（Q01–Q15，下拉选择；题目见“题目”工作表）</t>
+          <t>编号，已预填 D2b-001…；不用的行留着即可（没有 question_id 的行会被跳过）</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>layer</t>
+          <t>question_id</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>modelling = 列方程（S2）；execution = 解方程过程（S3）；answer = 只看最终答案（S4）</t>
+          <t>对应题库哪一题（Q01–Q15，下拉选择；题目见“题目”工作表）</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>variable_definition</t>
+          <t>layer</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>学生写的“设…”（modelling 可填；execution 可填；不写就留空）</t>
+          <t>modelling = 列方程（S2）；execution = 解方程过程（S3）；answer = 只看最终答案（S4）</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>equation</t>
+          <t>variable_definition</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>modelling：学生列的方程（必填）。execution：学生在 S2 列好的方程（选填；填了就从它开始检查第 1 行）</t>
+          <t>学生写的“设…”（modelling 可填；execution 可填；不写就留空）</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>steps</t>
+          <t>equation</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>execution：学生的解方程过程，一行一步（单元格内换行 Alt+Enter，或用 || 分隔）</t>
+          <t>modelling：学生列的方程（必填）。execution：学生在 S2 列好的方程（选填；填了就从它开始检查第 1 行）</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>final_answer_text</t>
+          <t>steps</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>answer：学生写的最终答案原文，例如“小明15岁，小华10岁”</t>
+          <t>execution：学生的解方程过程，一行一步（单元格内换行 Alt+Enter，或用 || 分隔）</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>reference_status</t>
+          <t>final_answer_text</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>你的判断：correct / incorrect / uncertain（两种解释都说得通）/ not_assessable（看不懂）</t>
+          <t>answer：学生写的最终答案原文，例如“小明15岁，小华10岁”</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>primary_error</t>
+          <t>reference_status</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>incorrect 时的主要错误类别 E1–E7（下拉）</t>
+          <t>你的判断：correct / incorrect / uncertain（两种解释都说得通）/ not_assessable（看不懂）</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>error_subtype</t>
+          <t>primary_error</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>只在 E4 时填 E4-01…E4-08（选填）</t>
+          <t>incorrect 时的主要错误类别 E1–E7（下拉）</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>secondary_errors</t>
+          <t>error_subtype</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>同时存在的其他独立错误，例如 E6;E7（多错误样本用）</t>
+          <t>只在 E4 时填 E4-01…E4-08（选填）</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>first_invalid_step</t>
+          <t>secondary_errors</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>execution 且有错时：steps 里第几行是第一个错的（从 1 数，只数 steps 单元格里的行）</t>
+          <t>同时存在的其他独立错误，例如 E6;E7（多错误样本用）</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>evidence_level</t>
+          <t>first_invalid_step</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>A 直接可见 / B 只从答案推断 / C 部分证据 / D 证据不足</t>
+          <t>execution 且有错时：steps 里第几行是第一个错的（从 1 数，只数 steps 单元格里的行）</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>tags</t>
+          <t>evidence_level</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>选填，分号分隔：equivalent_equation; alt_definition; alt_working; ambiguous_notation</t>
+          <t>A 直接可见 / B 只从答案推断 / C 部分证据 / D 证据不足</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>evidence</t>
+          <t>tags</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>作答里哪一处支持你的标注（原文摘录即可）</t>
+          <t>选填，分号分隔：equivalent_equation; alt_definition; alt_working; ambiguous_notation</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>evidence</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>备注（选填）</t>
+          <t>作答里哪一处支持你的标注（原文摘录即可）</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>备注（选填）</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
           <t>review_status</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>pending（写完还没复查）→ reviewed（复查定稿）；全部 reviewed 后才能冻结和正式运行</t>
         </is>

</xml_diff>

<commit_message>
Record D2b-009 correction and resolutions of second-annotator disagreements
</commit_message>
<xml_diff>
--- a/eval/d2b_cases.xlsx
+++ b/eval/d2b_cases.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="24750" windowHeight="12080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cases" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="题目" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="题目" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -2683,7 +2683,7 @@
       <c r="J23" s="2" t="n"/>
       <c r="K23" s="2" t="n"/>
       <c r="L23" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
@@ -2693,7 +2693,7 @@
       <c r="N23" s="2" t="n"/>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>作答依据：“设小华今年x岁，小明今年（x＋5）岁。”；最后一步x＝7错误；15÷2应为7.5。</t>
+          <t>2x＝25－5 之后写成 2x＝15,应为 2x＝20;第 3 步是第一个错误</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">

</xml_diff>